<commit_message>
jimbwal tole devithan nirmaan
</commit_message>
<xml_diff>
--- a/बजेट माग estimate/nagar bhaipari and estimate misc/जिम्वाल टोल देवीथान निर्माण/जिम्वाल टोल देवीथान निर्माण.xlsx
+++ b/बजेट माग estimate/nagar bhaipari and estimate misc/जिम्वाल टोल देवीथान निर्माण/जिम्वाल टोल देवीथान निर्माण.xlsx
@@ -1,10 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBC5B06F-95B4-4397-A08F-3A88158CBD2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20736" windowHeight="11040"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="estimate" sheetId="12" r:id="rId1"/>
@@ -39,7 +40,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="0">estimate!$A$1:$K$68</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">estimate!$1:$8</definedName>
   </definedNames>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -227,9 +228,6 @@
     <t>-MS square pipe of 3"*3" of 1.6mm thickness for horizontal purlin</t>
   </si>
   <si>
-    <t>-MS black pipe of 1.5"*1.5" of 1.6mm thickness for horizontal purlin</t>
-  </si>
-  <si>
     <t>-for masonary wall</t>
   </si>
   <si>
@@ -254,14 +252,17 @@
       <t>lhDjfn 6f]n b]jLyfg lgdf{0f l;l8 af6f]</t>
     </r>
   </si>
+  <si>
+    <t>-MS black pipe of 1.5"*1.5" of 2mm thickness for horizontal purlin</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
   <fonts count="15" x14ac:knownFonts="1">
     <font>
@@ -427,9 +428,9 @@
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
   </cellStyleXfs>
@@ -441,7 +442,7 @@
     <xf numFmtId="1" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -465,14 +466,14 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="43" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="9" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -491,7 +492,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -506,7 +507,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -534,7 +535,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -544,6 +545,12 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -581,20 +588,14 @@
     <xf numFmtId="2" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
-    <cellStyle name="Comma 2" xfId="3"/>
+    <cellStyle name="Comma 2" xfId="3" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="2"/>
-    <cellStyle name="Normal 3" xfId="5"/>
-    <cellStyle name="Percent 2" xfId="4"/>
+    <cellStyle name="Normal 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
+    <cellStyle name="Normal 3" xfId="5" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
+    <cellStyle name="Percent 2" xfId="4" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
@@ -610,7 +611,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Datasheet"/>
@@ -704,7 +705,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Datasheet"/>
@@ -763,7 +764,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink3.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Datasheet"/>
@@ -827,9 +828,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -867,9 +868,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -904,7 +905,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -939,7 +940,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1112,133 +1113,133 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K68"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="4.6640625" style="19" customWidth="1"/>
-    <col min="2" max="2" width="30.88671875" style="19" customWidth="1"/>
-    <col min="3" max="3" width="4.44140625" style="19" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.44140625" style="19" customWidth="1"/>
-    <col min="5" max="5" width="8.5546875" style="19" customWidth="1"/>
-    <col min="6" max="6" width="7.33203125" style="19" customWidth="1"/>
-    <col min="7" max="7" width="9.109375" style="19"/>
+    <col min="1" max="1" width="4.7109375" style="19" customWidth="1"/>
+    <col min="2" max="2" width="30.85546875" style="19" customWidth="1"/>
+    <col min="3" max="3" width="4.42578125" style="19" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.42578125" style="19" customWidth="1"/>
+    <col min="5" max="5" width="8.5703125" style="19" customWidth="1"/>
+    <col min="6" max="6" width="7.28515625" style="19" customWidth="1"/>
+    <col min="7" max="7" width="9.140625" style="19"/>
     <col min="8" max="8" width="5" style="19" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.5546875" style="19" customWidth="1"/>
-    <col min="10" max="10" width="10.6640625" style="19" bestFit="1" customWidth="1"/>
-    <col min="11" max="16384" width="9.109375" style="19"/>
+    <col min="9" max="9" width="9.5703125" style="19" customWidth="1"/>
+    <col min="10" max="10" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
+    <col min="11" max="16384" width="9.140625" style="19"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A1" s="46" t="s">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" s="48" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
-      <c r="F1" s="46"/>
-      <c r="G1" s="46"/>
-      <c r="H1" s="46"/>
-      <c r="I1" s="46"/>
-      <c r="J1" s="46"/>
-      <c r="K1" s="46"/>
-    </row>
-    <row r="2" spans="1:11" ht="22.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="47" t="s">
+      <c r="B1" s="48"/>
+      <c r="C1" s="48"/>
+      <c r="D1" s="48"/>
+      <c r="E1" s="48"/>
+      <c r="F1" s="48"/>
+      <c r="G1" s="48"/>
+      <c r="H1" s="48"/>
+      <c r="I1" s="48"/>
+      <c r="J1" s="48"/>
+      <c r="K1" s="48"/>
+    </row>
+    <row r="2" spans="1:11" ht="22.5" x14ac:dyDescent="0.25">
+      <c r="A2" s="49" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="47"/>
-      <c r="C2" s="47"/>
-      <c r="D2" s="47"/>
-      <c r="E2" s="47"/>
-      <c r="F2" s="47"/>
-      <c r="G2" s="47"/>
-      <c r="H2" s="47"/>
-      <c r="I2" s="47"/>
-      <c r="J2" s="47"/>
-      <c r="K2" s="47"/>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A3" s="48" t="s">
+      <c r="B2" s="49"/>
+      <c r="C2" s="49"/>
+      <c r="D2" s="49"/>
+      <c r="E2" s="49"/>
+      <c r="F2" s="49"/>
+      <c r="G2" s="49"/>
+      <c r="H2" s="49"/>
+      <c r="I2" s="49"/>
+      <c r="J2" s="49"/>
+      <c r="K2" s="49"/>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" s="50" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="48"/>
-      <c r="C3" s="48"/>
-      <c r="D3" s="48"/>
-      <c r="E3" s="48"/>
-      <c r="F3" s="48"/>
-      <c r="G3" s="48"/>
-      <c r="H3" s="48"/>
-      <c r="I3" s="48"/>
-      <c r="J3" s="48"/>
-      <c r="K3" s="48"/>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A4" s="48" t="s">
+      <c r="B3" s="50"/>
+      <c r="C3" s="50"/>
+      <c r="D3" s="50"/>
+      <c r="E3" s="50"/>
+      <c r="F3" s="50"/>
+      <c r="G3" s="50"/>
+      <c r="H3" s="50"/>
+      <c r="I3" s="50"/>
+      <c r="J3" s="50"/>
+      <c r="K3" s="50"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" s="50" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="48"/>
-      <c r="C4" s="48"/>
-      <c r="D4" s="48"/>
-      <c r="E4" s="48"/>
-      <c r="F4" s="48"/>
-      <c r="G4" s="48"/>
-      <c r="H4" s="48"/>
-      <c r="I4" s="48"/>
-      <c r="J4" s="48"/>
-      <c r="K4" s="48"/>
-    </row>
-    <row r="5" spans="1:11" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A5" s="49" t="s">
+      <c r="B4" s="50"/>
+      <c r="C4" s="50"/>
+      <c r="D4" s="50"/>
+      <c r="E4" s="50"/>
+      <c r="F4" s="50"/>
+      <c r="G4" s="50"/>
+      <c r="H4" s="50"/>
+      <c r="I4" s="50"/>
+      <c r="J4" s="50"/>
+      <c r="K4" s="50"/>
+    </row>
+    <row r="5" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A5" s="51" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="49"/>
-      <c r="C5" s="49"/>
-      <c r="D5" s="49"/>
-      <c r="E5" s="49"/>
-      <c r="F5" s="49"/>
-      <c r="G5" s="49"/>
-      <c r="H5" s="49"/>
-      <c r="I5" s="49"/>
-      <c r="J5" s="49"/>
-      <c r="K5" s="49"/>
-    </row>
-    <row r="6" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A6" s="44" t="s">
-        <v>61</v>
-      </c>
-      <c r="B6" s="44"/>
-      <c r="C6" s="44"/>
-      <c r="D6" s="44"/>
-      <c r="E6" s="44"/>
-      <c r="F6" s="44"/>
+      <c r="B5" s="51"/>
+      <c r="C5" s="51"/>
+      <c r="D5" s="51"/>
+      <c r="E5" s="51"/>
+      <c r="F5" s="51"/>
+      <c r="G5" s="51"/>
+      <c r="H5" s="51"/>
+      <c r="I5" s="51"/>
+      <c r="J5" s="51"/>
+      <c r="K5" s="51"/>
+    </row>
+    <row r="6" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A6" s="46" t="s">
+        <v>60</v>
+      </c>
+      <c r="B6" s="46"/>
+      <c r="C6" s="46"/>
+      <c r="D6" s="46"/>
+      <c r="E6" s="46"/>
+      <c r="F6" s="46"/>
       <c r="G6" s="10"/>
-      <c r="H6" s="45" t="s">
+      <c r="H6" s="47" t="s">
         <v>24</v>
       </c>
-      <c r="I6" s="45"/>
-      <c r="J6" s="45"/>
-      <c r="K6" s="45"/>
-    </row>
-    <row r="7" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A7" s="52" t="s">
+      <c r="I6" s="47"/>
+      <c r="J6" s="47"/>
+      <c r="K6" s="47"/>
+    </row>
+    <row r="7" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A7" s="54" t="s">
         <v>48</v>
       </c>
-      <c r="B7" s="52"/>
-      <c r="C7" s="52"/>
-      <c r="D7" s="52"/>
-      <c r="E7" s="52"/>
-      <c r="F7" s="52"/>
+      <c r="B7" s="54"/>
+      <c r="C7" s="54"/>
+      <c r="D7" s="54"/>
+      <c r="E7" s="54"/>
+      <c r="F7" s="54"/>
       <c r="G7" s="11"/>
-      <c r="H7" s="53" t="s">
+      <c r="H7" s="55" t="s">
         <v>53</v>
       </c>
-      <c r="I7" s="53"/>
-      <c r="J7" s="53"/>
-      <c r="K7" s="53"/>
-    </row>
-    <row r="8" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="I7" s="55"/>
+      <c r="J7" s="55"/>
+      <c r="K7" s="55"/>
+    </row>
+    <row r="8" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
         <v>5</v>
       </c>
@@ -1273,7 +1274,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:11" s="34" customFormat="1" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" s="34" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>1</v>
       </c>
@@ -1298,7 +1299,7 @@
       <c r="J9" s="38"/>
       <c r="K9" s="5"/>
     </row>
-    <row r="10" spans="1:11" s="34" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" s="34" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="16"/>
       <c r="B10" s="39" t="s">
         <v>54</v>
@@ -1326,7 +1327,7 @@
       <c r="J10" s="38"/>
       <c r="K10" s="27"/>
     </row>
-    <row r="11" spans="1:11" s="34" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" s="34" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="16"/>
       <c r="B11" s="39" t="s">
         <v>54</v>
@@ -1354,7 +1355,7 @@
       <c r="J11" s="38"/>
       <c r="K11" s="27"/>
     </row>
-    <row r="12" spans="1:11" s="34" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" s="34" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A12" s="16"/>
       <c r="B12" s="39" t="s">
         <v>55</v>
@@ -1382,7 +1383,7 @@
       <c r="J12" s="38"/>
       <c r="K12" s="27"/>
     </row>
-    <row r="13" spans="1:11" s="34" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" s="34" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="16"/>
       <c r="B13" s="39"/>
       <c r="C13" s="40">
@@ -1408,10 +1409,10 @@
       <c r="J13" s="38"/>
       <c r="K13" s="27"/>
     </row>
-    <row r="14" spans="1:11" s="34" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" s="34" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="16"/>
       <c r="B14" s="39" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C14" s="40">
         <v>2</v>
@@ -1421,22 +1422,22 @@
         <v>3.6574215178299299</v>
       </c>
       <c r="E14" s="9">
-        <v>2.88</v>
+        <v>2.2599999999999998</v>
       </c>
       <c r="F14" s="9">
         <f t="shared" ref="F14" si="6">PRODUCT(C14:E14)</f>
-        <v>21.066747942700395</v>
+        <v>16.531545260591283</v>
       </c>
       <c r="G14" s="9">
         <f t="shared" ref="G14" si="7">F14</f>
-        <v>21.066747942700395</v>
+        <v>16.531545260591283</v>
       </c>
       <c r="H14" s="38"/>
       <c r="I14" s="38"/>
       <c r="J14" s="38"/>
       <c r="K14" s="27"/>
     </row>
-    <row r="15" spans="1:11" s="34" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" s="34" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="16"/>
       <c r="B15" s="39"/>
       <c r="C15" s="40">
@@ -1447,22 +1448,22 @@
         <v>6.0957025297165499</v>
       </c>
       <c r="E15" s="9">
-        <v>2.88</v>
+        <v>2.2599999999999998</v>
       </c>
       <c r="F15" s="9">
         <f t="shared" ref="F15" si="8">PRODUCT(C15:E15)</f>
-        <v>17.555623285583664</v>
+        <v>13.776287717159402</v>
       </c>
       <c r="G15" s="9">
         <f t="shared" ref="G15" si="9">F15</f>
-        <v>17.555623285583664</v>
+        <v>13.776287717159402</v>
       </c>
       <c r="H15" s="38"/>
       <c r="I15" s="38"/>
       <c r="J15" s="38"/>
       <c r="K15" s="27"/>
     </row>
-    <row r="16" spans="1:11" s="34" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" s="34" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
       <c r="B16" s="39" t="s">
         <v>36</v>
@@ -1473,7 +1474,7 @@
       <c r="F16" s="5"/>
       <c r="G16" s="38">
         <f>SUM(G10:G15)</f>
-        <v>178.8844864370619</v>
+        <v>170.56994818652851</v>
       </c>
       <c r="H16" s="7" t="s">
         <v>37</v>
@@ -1483,11 +1484,11 @@
       </c>
       <c r="J16" s="38">
         <f>G16*I16</f>
-        <v>32648.207619628163</v>
+        <v>31130.721243523316</v>
       </c>
       <c r="K16" s="5"/>
     </row>
-    <row r="17" spans="1:11" s="34" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" s="34" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2"/>
       <c r="B17" s="39" t="s">
         <v>38</v>
@@ -1501,11 +1502,11 @@
       <c r="I17" s="6"/>
       <c r="J17" s="38">
         <f>0.13*G16*(1871.42/18.94)</f>
-        <v>2297.7740617236554</v>
+        <v>2190.9736861974825</v>
       </c>
       <c r="K17" s="5"/>
     </row>
-    <row r="18" spans="1:11" s="34" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" s="34" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2"/>
       <c r="B18" s="39"/>
       <c r="C18" s="3"/>
@@ -1518,7 +1519,7 @@
       <c r="J18" s="38"/>
       <c r="K18" s="5"/>
     </row>
-    <row r="19" spans="1:11" s="34" customFormat="1" ht="30" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" s="34" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
         <v>2</v>
       </c>
@@ -1535,7 +1536,7 @@
       <c r="J19" s="38"/>
       <c r="K19" s="5"/>
     </row>
-    <row r="20" spans="1:11" s="34" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" s="34" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2"/>
       <c r="B20" s="39" t="s">
         <v>49</v>
@@ -1561,7 +1562,7 @@
       <c r="J20" s="38"/>
       <c r="K20" s="5"/>
     </row>
-    <row r="21" spans="1:11" s="34" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" s="34" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2"/>
       <c r="B21" s="39" t="s">
         <v>36</v>
@@ -1586,7 +1587,7 @@
       </c>
       <c r="K21" s="5"/>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="16"/>
       <c r="B22" s="32" t="s">
         <v>40</v>
@@ -1604,7 +1605,7 @@
       </c>
       <c r="K22" s="17"/>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="16"/>
       <c r="B23" s="32" t="s">
         <v>41</v>
@@ -1622,7 +1623,7 @@
       </c>
       <c r="K23" s="17"/>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="16"/>
       <c r="B24" s="32" t="s">
         <v>42</v>
@@ -1640,7 +1641,7 @@
       </c>
       <c r="K24" s="17"/>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="16"/>
       <c r="B25" s="32" t="s">
         <v>43</v>
@@ -1658,7 +1659,7 @@
       </c>
       <c r="K25" s="17"/>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="16"/>
       <c r="B26" s="32"/>
       <c r="C26" s="17"/>
@@ -1671,7 +1672,7 @@
       <c r="J26" s="18"/>
       <c r="K26" s="17"/>
     </row>
-    <row r="27" spans="1:11" ht="129.6" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:11" ht="150" x14ac:dyDescent="0.25">
       <c r="A27" s="16">
         <v>3</v>
       </c>
@@ -1688,10 +1689,10 @@
       <c r="J27" s="18"/>
       <c r="K27" s="17"/>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="16"/>
       <c r="B28" s="32" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C28" s="17">
         <v>1</v>
@@ -1715,7 +1716,7 @@
       <c r="J28" s="18"/>
       <c r="K28" s="17"/>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="16"/>
       <c r="B29" s="32" t="s">
         <v>47</v>
@@ -1742,7 +1743,7 @@
       <c r="J29" s="18"/>
       <c r="K29" s="17"/>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="16"/>
       <c r="B30" s="32" t="str">
         <f>B35</f>
@@ -1772,7 +1773,7 @@
       <c r="J30" s="18"/>
       <c r="K30" s="17"/>
     </row>
-    <row r="31" spans="1:11" s="34" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:11" s="34" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2"/>
       <c r="B31" s="39" t="s">
         <v>36</v>
@@ -1797,7 +1798,7 @@
       </c>
       <c r="K31" s="5"/>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" s="16"/>
       <c r="B32" s="32"/>
       <c r="C32" s="17"/>
@@ -1810,7 +1811,7 @@
       <c r="J32" s="18"/>
       <c r="K32" s="17"/>
     </row>
-    <row r="33" spans="1:11" ht="90" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:11" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="16">
         <v>4</v>
       </c>
@@ -1827,7 +1828,7 @@
       <c r="J33" s="18"/>
       <c r="K33" s="17"/>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" s="16"/>
       <c r="B34" s="32" t="str">
         <f>B41</f>
@@ -1857,7 +1858,7 @@
       <c r="J34" s="18"/>
       <c r="K34" s="17"/>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" s="16"/>
       <c r="B35" s="32" t="s">
         <v>51</v>
@@ -1885,7 +1886,7 @@
       <c r="J35" s="18"/>
       <c r="K35" s="17"/>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" s="16"/>
       <c r="B36" s="32" t="str">
         <f>B29</f>
@@ -1915,7 +1916,7 @@
       <c r="J36" s="18"/>
       <c r="K36" s="17"/>
     </row>
-    <row r="37" spans="1:11" s="34" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:11" s="34" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="2"/>
       <c r="B37" s="39" t="s">
         <v>36</v>
@@ -1940,7 +1941,7 @@
       </c>
       <c r="K37" s="5"/>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" s="16"/>
       <c r="B38" s="32" t="s">
         <v>29</v>
@@ -1958,7 +1959,7 @@
       </c>
       <c r="K38" s="17"/>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" s="16"/>
       <c r="B39" s="41"/>
       <c r="C39" s="17"/>
@@ -1971,7 +1972,7 @@
       <c r="J39" s="18"/>
       <c r="K39" s="17"/>
     </row>
-    <row r="40" spans="1:11" ht="83.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:11" ht="83.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="16">
         <v>5</v>
       </c>
@@ -1988,7 +1989,7 @@
       <c r="J40" s="17"/>
       <c r="K40" s="17"/>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" s="16"/>
       <c r="B41" s="32" t="str">
         <f>B52</f>
@@ -2018,22 +2019,22 @@
       <c r="J41" s="18"/>
       <c r="K41" s="17"/>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" s="16"/>
       <c r="B42" s="32" t="str">
-        <f>B35</f>
+        <f t="shared" ref="B42:E43" si="14">B35</f>
         <v>-for plinth</v>
       </c>
       <c r="C42" s="17">
-        <f>C35</f>
+        <f t="shared" si="14"/>
         <v>1</v>
       </c>
       <c r="D42" s="33">
-        <f>D35</f>
+        <f t="shared" si="14"/>
         <v>5.486132276744895</v>
       </c>
       <c r="E42" s="33">
-        <f>E35</f>
+        <f t="shared" si="14"/>
         <v>3.047851264858275</v>
       </c>
       <c r="F42" s="33">
@@ -2048,22 +2049,22 @@
       <c r="J42" s="18"/>
       <c r="K42" s="17"/>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" s="16"/>
       <c r="B43" s="32" t="str">
-        <f>B36</f>
+        <f t="shared" si="14"/>
         <v>-for footing of vertical post</v>
       </c>
       <c r="C43" s="17">
-        <f>C36</f>
+        <f t="shared" si="14"/>
         <v>6</v>
       </c>
       <c r="D43" s="33">
-        <f>D36</f>
+        <f t="shared" si="14"/>
         <v>0.3</v>
       </c>
       <c r="E43" s="33">
-        <f>E36</f>
+        <f t="shared" si="14"/>
         <v>0.3</v>
       </c>
       <c r="F43" s="33">
@@ -2079,7 +2080,7 @@
       <c r="J43" s="18"/>
       <c r="K43" s="17"/>
     </row>
-    <row r="44" spans="1:11" s="34" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:11" s="34" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="2"/>
       <c r="B44" s="39" t="s">
         <v>36</v>
@@ -2104,7 +2105,7 @@
       </c>
       <c r="K44" s="5"/>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" s="16"/>
       <c r="B45" s="32" t="s">
         <v>26</v>
@@ -2122,7 +2123,7 @@
       </c>
       <c r="K45" s="17"/>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" s="16"/>
       <c r="B46" s="32" t="s">
         <v>27</v>
@@ -2140,7 +2141,7 @@
       </c>
       <c r="K46" s="17"/>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" s="16"/>
       <c r="B47" s="32" t="s">
         <v>28</v>
@@ -2158,7 +2159,7 @@
       </c>
       <c r="K47" s="17"/>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" s="16"/>
       <c r="B48" s="32" t="s">
         <v>46</v>
@@ -2176,7 +2177,7 @@
       </c>
       <c r="K48" s="17"/>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" s="16"/>
       <c r="B49" s="32" t="s">
         <v>30</v>
@@ -2194,7 +2195,7 @@
       </c>
       <c r="K49" s="17"/>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" s="16"/>
       <c r="B50" s="32"/>
       <c r="C50" s="17"/>
@@ -2207,12 +2208,12 @@
       <c r="J50" s="18"/>
       <c r="K50" s="17"/>
     </row>
-    <row r="51" spans="1:11" ht="109.2" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:11" ht="110.25" x14ac:dyDescent="0.25">
       <c r="A51" s="16">
-        <v>4</v>
-      </c>
-      <c r="B51" s="57" t="s">
-        <v>58</v>
+        <v>6</v>
+      </c>
+      <c r="B51" s="44" t="s">
+        <v>57</v>
       </c>
       <c r="C51" s="17"/>
       <c r="D51" s="17"/>
@@ -2224,7 +2225,7 @@
       <c r="J51" s="17"/>
       <c r="K51" s="17"/>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" s="16"/>
       <c r="B52" s="32" t="str">
         <f>B28</f>
@@ -2252,10 +2253,10 @@
       <c r="J52" s="17"/>
       <c r="K52" s="17"/>
     </row>
-    <row r="53" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="2"/>
-      <c r="B53" s="58" t="s">
-        <v>59</v>
+      <c r="B53" s="45" t="s">
+        <v>58</v>
       </c>
       <c r="C53" s="3"/>
       <c r="D53" s="4"/>
@@ -2266,7 +2267,7 @@
         <v>2.2218835720816825</v>
       </c>
       <c r="H53" s="7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="I53" s="6">
         <v>8987.83</v>
@@ -2277,7 +2278,7 @@
       </c>
       <c r="K53" s="5"/>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" s="16"/>
       <c r="B54" s="32" t="s">
         <v>26</v>
@@ -2295,7 +2296,7 @@
       </c>
       <c r="K54" s="17"/>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" s="16"/>
       <c r="B55" s="32" t="s">
         <v>27</v>
@@ -2313,7 +2314,7 @@
       </c>
       <c r="K55" s="17"/>
     </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" s="16"/>
       <c r="B56" s="32" t="s">
         <v>29</v>
@@ -2331,7 +2332,7 @@
       </c>
       <c r="K56" s="17"/>
     </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" s="16"/>
       <c r="B57" s="32" t="s">
         <v>30</v>
@@ -2349,7 +2350,7 @@
       </c>
       <c r="K57" s="17"/>
     </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" s="16"/>
       <c r="B58" s="17"/>
       <c r="C58" s="17"/>
@@ -2362,9 +2363,9 @@
       <c r="J58" s="17"/>
       <c r="K58" s="17"/>
     </row>
-    <row r="59" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="2">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B59" s="1" t="s">
         <v>16</v>
@@ -2376,7 +2377,7 @@
       <c r="E59" s="5"/>
       <c r="F59" s="5"/>
       <c r="G59" s="7">
-        <f t="shared" ref="G59" si="14">PRODUCT(C59:F59)</f>
+        <f t="shared" ref="G59" si="15">PRODUCT(C59:F59)</f>
         <v>1</v>
       </c>
       <c r="H59" s="7" t="s">
@@ -2391,7 +2392,7 @@
       </c>
       <c r="K59" s="5"/>
     </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" s="2"/>
       <c r="B60" s="8"/>
       <c r="C60" s="3"/>
@@ -2404,7 +2405,7 @@
       <c r="J60" s="18"/>
       <c r="K60" s="5"/>
     </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" s="21"/>
       <c r="B61" s="22" t="s">
         <v>19</v>
@@ -2418,20 +2419,20 @@
       <c r="I61" s="18"/>
       <c r="J61" s="18">
         <f>SUM(J9:J59)</f>
-        <v>120056.07114071168</v>
+        <v>118431.78438908067</v>
       </c>
       <c r="K61" s="25"/>
     </row>
-    <row r="63" spans="1:11" s="20" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:11" s="20" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A63" s="26"/>
       <c r="B63" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="C63" s="50">
+      <c r="C63" s="52">
         <f>J61</f>
-        <v>120056.07114071168</v>
-      </c>
-      <c r="D63" s="51"/>
+        <v>118431.78438908067</v>
+      </c>
+      <c r="D63" s="53"/>
       <c r="E63" s="9">
         <v>100</v>
       </c>
@@ -2442,66 +2443,66 @@
       <c r="J63" s="30"/>
       <c r="K63" s="31"/>
     </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B64" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="C64" s="54">
+      <c r="C64" s="56">
         <v>100000</v>
       </c>
-      <c r="D64" s="55"/>
+      <c r="D64" s="57"/>
       <c r="E64" s="9"/>
     </row>
-    <row r="65" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="65" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B65" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="C65" s="54">
+      <c r="C65" s="56">
         <f>C64-C67-C68</f>
         <v>95000</v>
       </c>
-      <c r="D65" s="55"/>
+      <c r="D65" s="57"/>
       <c r="E65" s="9">
         <f>C65/C63*100</f>
-        <v>79.129692565614022</v>
-      </c>
-    </row>
-    <row r="66" spans="2:5" x14ac:dyDescent="0.3">
+        <v>80.214952843992563</v>
+      </c>
+    </row>
+    <row r="66" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B66" s="27" t="s">
         <v>31</v>
       </c>
-      <c r="C66" s="56">
+      <c r="C66" s="58">
         <f>C63-C65</f>
-        <v>25056.071140711676</v>
-      </c>
-      <c r="D66" s="56"/>
+        <v>23431.784389080669</v>
+      </c>
+      <c r="D66" s="58"/>
       <c r="E66" s="9">
         <f>100-E65</f>
-        <v>20.870307434385978</v>
-      </c>
-    </row>
-    <row r="67" spans="2:5" x14ac:dyDescent="0.3">
+        <v>19.785047156007437</v>
+      </c>
+    </row>
+    <row r="67" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B67" s="27" t="s">
         <v>22</v>
       </c>
-      <c r="C67" s="50">
+      <c r="C67" s="52">
         <f>C64*0.03</f>
         <v>3000</v>
       </c>
-      <c r="D67" s="51"/>
+      <c r="D67" s="53"/>
       <c r="E67" s="9">
         <v>3</v>
       </c>
     </row>
-    <row r="68" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="68" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B68" s="27" t="s">
         <v>23</v>
       </c>
-      <c r="C68" s="50">
+      <c r="C68" s="52">
         <f>C64*0.02</f>
         <v>2000</v>
       </c>
-      <c r="D68" s="51"/>
+      <c r="D68" s="53"/>
       <c r="E68" s="9">
         <v>2</v>
       </c>

</xml_diff>